<commit_message>
Modified column names and added notes for clarification to excel sheets
</commit_message>
<xml_diff>
--- a/raw-data/sample_info_snRNAseq/2024-01-31_ERC_chromium_round_1_sequencing_summary.xlsx
+++ b/raw-data/sample_info_snRNAseq/2024-01-31_ERC_chromium_round_1_sequencing_summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/vs/jsj0ztfs21v1pxhnd7gs3vkr0000gn/T/ch.sudo.cyberduck/editor-796f2507-b176-4189-be46-ee4f12ac67b6/bd05a3abaeafc2f65e6f0293bbd8bc49/738915530/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/vs/jsj0ztfs21v1pxhnd7gs3vkr0000gn/T/ch.sudo.cyberduck/editor-796f2507-b176-4189-be46-ee4f12ac67b6/bd05a3abaeafc2f65e6f0293bbd8bc49/-453717847/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF3AC5D6-E534-A644-BA8E-361A2C701C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071EC705-D71A-F943-BE2F-987F62A7AC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20920" windowHeight="12560" xr2:uid="{CD1FF015-2F3F-48C0-BAF6-738726850051}"/>
+    <workbookView xWindow="31400" yWindow="5400" windowWidth="22380" windowHeight="12880" xr2:uid="{CD1FF015-2F3F-48C0-BAF6-738726850051}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="50">
   <si>
     <t>Sample #</t>
   </si>
@@ -168,13 +168,31 @@
   </si>
   <si>
     <t>TTGAGTATAG</t>
+  </si>
+  <si>
+    <t>cDNA Dilution Factor</t>
+  </si>
+  <si>
+    <t>Lib Dilution Factor</t>
+  </si>
+  <si>
+    <t>Experimental Round</t>
+  </si>
+  <si>
+    <t>Sequencing Round</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>some samples had the same index...so they couldn't be sequenced together.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -205,6 +223,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1D1C1D"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -220,7 +253,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -243,12 +276,47 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -270,6 +338,20 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -899,32 +981,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB585CF4-08FC-4734-A306-FBD8539CEC9B}">
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" customWidth="1"/>
     <col min="2" max="2" width="14.5" style="8" customWidth="1"/>
-    <col min="3" max="5" width="8.83203125" style="8"/>
-    <col min="6" max="6" width="12.1640625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" style="8" customWidth="1"/>
-    <col min="8" max="8" width="16.1640625" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" style="2" customWidth="1"/>
-    <col min="10" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="13.5" style="2" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="13.5" customWidth="1"/>
-    <col min="16" max="16" width="14.1640625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="11.83203125" customWidth="1"/>
-    <col min="18" max="18" width="16.5" style="2" customWidth="1"/>
-    <col min="19" max="19" width="17.6640625" customWidth="1"/>
-    <col min="20" max="20" width="18.1640625" customWidth="1"/>
-    <col min="21" max="21" width="17.83203125" customWidth="1"/>
-    <col min="22" max="22" width="18.5" customWidth="1"/>
-    <col min="23" max="23" width="18.1640625" customWidth="1"/>
+    <col min="3" max="6" width="8.83203125" style="8"/>
+    <col min="7" max="7" width="12.1640625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" style="8" customWidth="1"/>
+    <col min="9" max="9" width="16.1640625" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" style="2" customWidth="1"/>
+    <col min="11" max="12" width="12.6640625" customWidth="1"/>
+    <col min="13" max="13" width="13.5" style="2" customWidth="1"/>
+    <col min="14" max="14" width="13.33203125" style="2" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
+    <col min="16" max="16" width="13.5" customWidth="1"/>
+    <col min="17" max="17" width="14.1640625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1"/>
+    <col min="19" max="19" width="16.5" style="2" customWidth="1"/>
+    <col min="20" max="20" width="17.6640625" customWidth="1"/>
+    <col min="21" max="21" width="18.1640625" customWidth="1"/>
+    <col min="22" max="22" width="17.83203125" customWidth="1"/>
+    <col min="23" max="23" width="18.5" customWidth="1"/>
+    <col min="24" max="24" width="18.1640625" customWidth="1"/>
+    <col min="25" max="25" width="59" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="34" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -935,67 +1018,73 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="E1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>6</v>
-      </c>
       <c r="K1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="Q1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="14" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="Y1" s="18" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -1008,69 +1097,73 @@
       <c r="D2" s="6">
         <v>1</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="6">
+        <v>1</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="6">
+      <c r="G2" s="6">
         <v>14000</v>
       </c>
-      <c r="G2" s="6">
+      <c r="H2" s="6">
         <v>9000</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="1">
         <v>11</v>
       </c>
-      <c r="I2" s="5">
+      <c r="J2" s="5">
         <v>806.56</v>
       </c>
-      <c r="J2" s="1">
+      <c r="K2" s="1">
         <v>2</v>
       </c>
-      <c r="K2" s="9">
-        <f t="shared" ref="K2:K4" si="0">I2*J2</f>
+      <c r="L2" s="9">
+        <f t="shared" ref="L2:L4" si="0">J2*K2</f>
         <v>1613.12</v>
       </c>
-      <c r="L2" s="10">
-        <f t="shared" ref="L2:L4" si="1">(K2*40)/1000</f>
+      <c r="M2" s="10">
+        <f t="shared" ref="M2:M4" si="1">(L2*40)/1000</f>
         <v>64.524799999999999</v>
       </c>
-      <c r="M2" s="10">
-        <f t="shared" ref="M2:M4" si="2">L2*0.25</f>
+      <c r="N2" s="10">
+        <f t="shared" ref="N2:N4" si="2">M2*0.25</f>
         <v>16.1312</v>
       </c>
-      <c r="N2" s="1">
+      <c r="O2" s="1">
         <v>15</v>
       </c>
-      <c r="O2" s="1">
+      <c r="P2" s="1">
         <v>490</v>
       </c>
-      <c r="P2" s="5">
+      <c r="Q2" s="5">
         <v>1090.83</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="R2" s="1">
         <v>10</v>
       </c>
-      <c r="R2" s="10">
-        <f t="shared" ref="R2:R4" si="3">P2*Q2</f>
+      <c r="S2" s="10">
+        <f t="shared" ref="S2:S4" si="3">Q2*R2</f>
         <v>10908.3</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="W2" s="1">
+      <c r="X2" s="15">
         <v>420</v>
       </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="Y2" s="16"/>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>26</v>
       </c>
@@ -1083,69 +1176,73 @@
       <c r="D3" s="6">
         <v>1</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="6"/>
+      <c r="F3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="6">
+      <c r="G3" s="6">
         <v>14000</v>
       </c>
-      <c r="G3" s="6">
+      <c r="H3" s="6">
         <v>9000</v>
       </c>
-      <c r="H3" s="1">
+      <c r="I3" s="1">
         <v>11</v>
       </c>
-      <c r="I3" s="5">
+      <c r="J3" s="5">
         <v>1249.4100000000001</v>
       </c>
-      <c r="J3" s="1">
+      <c r="K3" s="1">
         <v>2</v>
       </c>
-      <c r="K3" s="9">
+      <c r="L3" s="9">
         <f t="shared" si="0"/>
         <v>2498.8200000000002</v>
       </c>
-      <c r="L3" s="10">
+      <c r="M3" s="10">
         <f t="shared" si="1"/>
         <v>99.952799999999996</v>
       </c>
-      <c r="M3" s="10">
+      <c r="N3" s="10">
         <f t="shared" si="2"/>
         <v>24.988199999999999</v>
       </c>
-      <c r="N3" s="1">
+      <c r="O3" s="1">
         <v>14</v>
       </c>
-      <c r="O3" s="1">
+      <c r="P3" s="1">
         <v>463</v>
       </c>
-      <c r="P3" s="5">
+      <c r="Q3" s="5">
         <v>1698.92</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="R3" s="1">
         <v>13</v>
       </c>
-      <c r="R3" s="10">
+      <c r="S3" s="10">
         <f t="shared" si="3"/>
         <v>22085.96</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="T3" t="s">
+      <c r="U3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="W3" s="1">
+      <c r="X3" s="15">
         <v>420</v>
       </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="Y3" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>27</v>
       </c>
@@ -1158,94 +1255,99 @@
       <c r="D4" s="6">
         <v>1</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="6"/>
+      <c r="F4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>14000</v>
       </c>
-      <c r="G4" s="6">
+      <c r="H4" s="6">
         <v>9000</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="1">
         <v>11</v>
       </c>
-      <c r="I4" s="5">
+      <c r="J4" s="5">
         <v>1127.5999999999999</v>
       </c>
-      <c r="J4" s="1">
+      <c r="K4" s="1">
         <v>2</v>
       </c>
-      <c r="K4" s="9">
+      <c r="L4" s="9">
         <f t="shared" si="0"/>
         <v>2255.1999999999998</v>
       </c>
-      <c r="L4" s="10">
+      <c r="M4" s="10">
         <f t="shared" si="1"/>
         <v>90.207999999999998</v>
       </c>
-      <c r="M4" s="10">
+      <c r="N4" s="10">
         <f t="shared" si="2"/>
         <v>22.552</v>
       </c>
-      <c r="N4" s="1">
+      <c r="O4" s="1">
         <v>14</v>
       </c>
-      <c r="O4" s="1">
+      <c r="P4" s="1">
         <v>456</v>
       </c>
-      <c r="P4" s="5">
+      <c r="Q4" s="5">
         <v>1425.87</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="R4" s="1">
         <v>10</v>
       </c>
-      <c r="R4" s="10">
+      <c r="S4" s="10">
         <f t="shared" si="3"/>
         <v>14258.699999999999</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="T4" t="s">
+      <c r="U4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="V4" t="s">
+      <c r="W4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="W4" s="1">
+      <c r="X4" s="15">
         <v>420</v>
       </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="1"/>
-      <c r="U5" s="1"/>
-      <c r="V5" s="1"/>
-      <c r="W5" s="1"/>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="Y4" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="13"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -1253,24 +1355,25 @@
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="1"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="5"/>
       <c r="K6" s="1"/>
-      <c r="L6" s="5"/>
+      <c r="L6" s="1"/>
       <c r="M6" s="5"/>
-      <c r="N6" s="1"/>
+      <c r="N6" s="5"/>
       <c r="O6" s="1"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="5"/>
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X6" s="1"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1278,24 +1381,25 @@
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="1"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="5"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="5"/>
+      <c r="L7" s="1"/>
       <c r="M7" s="5"/>
-      <c r="N7" s="1"/>
+      <c r="N7" s="5"/>
       <c r="O7" s="1"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="5"/>
-      <c r="S7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="5"/>
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1"/>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X7" s="1"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1303,24 +1407,25 @@
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="1"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="5"/>
       <c r="K8" s="1"/>
-      <c r="L8" s="5"/>
+      <c r="L8" s="1"/>
       <c r="M8" s="5"/>
-      <c r="N8" s="1"/>
+      <c r="N8" s="5"/>
       <c r="O8" s="1"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="5"/>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X8" s="1"/>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1328,24 +1433,25 @@
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="1"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="5"/>
       <c r="K9" s="1"/>
-      <c r="L9" s="5"/>
+      <c r="L9" s="1"/>
       <c r="M9" s="5"/>
-      <c r="N9" s="1"/>
+      <c r="N9" s="5"/>
       <c r="O9" s="1"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="1"/>
+      <c r="S9" s="5"/>
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X9" s="1"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1353,24 +1459,25 @@
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="1"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="5"/>
       <c r="K10" s="1"/>
-      <c r="L10" s="5"/>
+      <c r="L10" s="1"/>
       <c r="M10" s="5"/>
-      <c r="N10" s="1"/>
+      <c r="N10" s="5"/>
       <c r="O10" s="1"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="1"/>
+      <c r="S10" s="5"/>
       <c r="T10" s="1"/>
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1"/>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X10" s="1"/>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1378,22 +1485,23 @@
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="1"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="5"/>
       <c r="K11" s="1"/>
-      <c r="L11" s="5"/>
+      <c r="L11" s="1"/>
       <c r="M11" s="5"/>
-      <c r="N11" s="1"/>
+      <c r="N11" s="5"/>
       <c r="O11" s="1"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="1"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="1"/>
+      <c r="S11" s="5"/>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
+      <c r="X11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>